<commit_message>
adding updated manual doc
</commit_message>
<xml_diff>
--- a/ManualDoc/Manual_Testing_Templates.xlsx
+++ b/ManualDoc/Manual_Testing_Templates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42f80ba52e01bcc9/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/42f80ba52e01bcc9/Desktop/final_project (5)/final_project (4)/final_project (2)/final_project/ManualDoc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="526" documentId="11_F7E64891378C4214A6B1EBC7DCE160856676FAD4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B967AAD0-9D67-442C-B2E8-13E358460EC7}"/>
+  <xr:revisionPtr revIDLastSave="550" documentId="11_F7E64891378C4214A6B1EBC7DCE160856676FAD4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FC2B905-76E2-4ED1-8B2A-799E88ABC37F}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Guidance &amp; Instructions" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="355">
   <si>
     <t>MANUAL TESTING DOCUMENTATION GUIDE</t>
   </si>
@@ -1110,6 +1110,24 @@
   </si>
   <si>
     <t>Build is not ready for release due to open high and medium severity defects affecting core functionality and user experience.</t>
+  </si>
+  <si>
+    <t>DEF-003</t>
+  </si>
+  <si>
+    <t>No bulk delete option for notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Application does not support selecting multiple notes for deletion; user must delete notes one by one, making the process time-consuming and less user-friendly</t>
+  </si>
+  <si>
+    <t>Dev-User3</t>
+  </si>
+  <si>
+    <t>UI enhancement required for better UX</t>
+  </si>
+  <si>
+    <t>Manual Tester, Automation Tester</t>
   </si>
 </sst>
 </file>
@@ -1279,10 +1297,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2049,13 +2063,16 @@
       <c r="A34" t="s">
         <v>76</v>
       </c>
+      <c r="B34" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>169</v>
+        <v>354</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -3327,7 +3344,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3435,6 +3452,38 @@
       </c>
       <c r="J3" s="7" t="s">
         <v>345</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="I4" s="15">
+        <v>46147</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -3550,7 +3599,7 @@
         <v>156</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -3574,7 +3623,7 @@
         <v>159</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -3590,7 +3639,7 @@
         <v>161</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>